<commit_message>
New data with timings for random polynomial rMEPs. Tools for figures for the paper.
</commit_message>
<xml_diff>
--- a/Comparison_linear_RMEP.xlsx
+++ b/Comparison_linear_RMEP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\MEP\RMEP_homotopy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13AFCD8C-DC77-4F5C-8BA9-6442BBA3F318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E79BD728-A493-450D-B8F1-C8E3E0E2AACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16200" yWindow="1416" windowWidth="23124" windowHeight="15936" activeTab="2" xr2:uid="{A4011660-FB7A-4DB9-A678-D73B0BBE67FE}"/>
+    <workbookView xWindow="240" yWindow="276" windowWidth="30312" windowHeight="17028" xr2:uid="{A4011660-FB7A-4DB9-A678-D73B0BBE67FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Times" sheetId="1" r:id="rId1"/>
@@ -1748,7 +1748,7 @@
     </row>
     <row r="11" spans="1:56" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B11">
         <v>36</v>

</xml_diff>